<commit_message>
feat: add Admission Date column to student import
- Column 12 (L) = Admission Date (DD/MM/YYYY); used for inquiry_date
  and confirmed_date on the admission record
- Leave blank to default to today; invalid format gets a warning and
  falls back to today
- Roll numbers will now be ordered by realistic admission dates rather
  than all having the same import date
- All 11 class import files regenerated with class-appropriate random
  admission dates (Nursery Dec 2024 – Feb 2025 → Class 8 Dec 2015 –
  Feb 2016, with ~20% late/transfer date variation per class)
- Preview table shows Adm. Date column; instructions sheet updated

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schoolDocs/Class1_ImportReady.xlsx
+++ b/schoolDocs/Class1_ImportReady.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="99">
   <si>
     <t>Sr No</t>
   </si>
@@ -50,6 +50,9 @@
     <t>Already Collected (Rs)</t>
   </si>
   <si>
+    <t>Admission Date (DD/MM/YYYY)</t>
+  </si>
+  <si>
     <t>Village</t>
   </si>
   <si>
@@ -92,6 +95,9 @@
     <t>rte</t>
   </si>
   <si>
+    <t>13/01/2023</t>
+  </si>
+  <si>
     <t>Kedgaon</t>
   </si>
   <si>
@@ -110,6 +116,9 @@
     <t>Om Sunil Ingle</t>
   </si>
   <si>
+    <t>10/02/2023</t>
+  </si>
+  <si>
     <t>Wakdapul</t>
   </si>
   <si>
@@ -125,12 +134,18 @@
     <t>general</t>
   </si>
   <si>
+    <t>02/01/2025</t>
+  </si>
+  <si>
     <t>Boripardhi</t>
   </si>
   <si>
     <t>Siddhiraj Baburao Kolpe</t>
   </si>
   <si>
+    <t>16/12/2024</t>
+  </si>
+  <si>
     <t>Keskarvasti</t>
   </si>
   <si>
@@ -146,12 +161,18 @@
     <t>Kartik D Nevase</t>
   </si>
   <si>
+    <t>08/01/2025</t>
+  </si>
+  <si>
     <t>Works at mobile shop</t>
   </si>
   <si>
     <t>Soham Amol Pathare</t>
   </si>
   <si>
+    <t>20/12/2022</t>
+  </si>
+  <si>
     <t>Works at Sayadri</t>
   </si>
   <si>
@@ -161,6 +182,9 @@
     <t>discount</t>
   </si>
   <si>
+    <t>18/01/2025</t>
+  </si>
+  <si>
     <t>Chaufula</t>
   </si>
   <si>
@@ -179,6 +203,9 @@
     <t>coc</t>
   </si>
   <si>
+    <t>28/01/2023</t>
+  </si>
+  <si>
     <t>Kasurdi</t>
   </si>
   <si>
@@ -191,31 +218,49 @@
     <t>Samarthraj Ajithkumar Desinayak</t>
   </si>
   <si>
+    <t>15/01/2025</t>
+  </si>
+  <si>
     <t>75% discount on boys ₹16200 = ₹4050 payable — collected ₹2000 (partial). Verify discount %.</t>
   </si>
   <si>
     <t>Jivnath Navnath Pawar</t>
   </si>
   <si>
+    <t>18/12/2022</t>
+  </si>
+  <si>
     <t>CoC student — full ₹16200 collected</t>
   </si>
   <si>
     <t>Vedansh Popat Yale</t>
   </si>
   <si>
-    <t>Partial payment — ₹7000 of ₹16200 collected</t>
+    <t>31/01/2025</t>
+  </si>
+  <si>
+    <t>Partial — ₹7000 of ₹16200 collected</t>
   </si>
   <si>
     <t>Swaraj Lakshman Kashid</t>
   </si>
   <si>
+    <t>19/01/2025</t>
+  </si>
+  <si>
     <t>Yash Raju Sarode</t>
   </si>
   <si>
+    <t>07/01/2023</t>
+  </si>
+  <si>
     <t>Aryan Ganesh Pawar</t>
   </si>
   <si>
-    <t>Partial payment — ₹9450 of ₹16200 collected</t>
+    <t>22/12/2022</t>
+  </si>
+  <si>
+    <t>Partial — ₹9450 of ₹16200 collected</t>
   </si>
   <si>
     <t>Chaitrali Rahul Chaudhari</t>
@@ -224,15 +269,24 @@
     <t>female</t>
   </si>
   <si>
-    <t>Partial payment — ₹5000 of ₹12200 collected</t>
+    <t>07/01/2025</t>
+  </si>
+  <si>
+    <t>Partial — ₹5000 of ₹12200 collected</t>
   </si>
   <si>
     <t>Shravani Amit Kale</t>
   </si>
   <si>
+    <t>08/02/2025</t>
+  </si>
+  <si>
     <t>Divya Dada Kokre</t>
   </si>
   <si>
+    <t>24/12/2024</t>
+  </si>
+  <si>
     <t>Shepherd</t>
   </si>
   <si>
@@ -240,6 +294,9 @@
   </si>
   <si>
     <t>Blessing Deepak Tujare</t>
+  </si>
+  <si>
+    <t>07/02/2023</t>
   </si>
   <si>
     <t>Bhandgaon</t>
@@ -291,7 +348,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -316,6 +373,12 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5EAD0"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -329,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
@@ -338,6 +401,9 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="2" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="5" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
@@ -640,7 +706,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="9.283" bestFit="true" customWidth="true" style="0"/>
@@ -654,18 +720,19 @@
     <col min="9" max="9" width="15.139" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="24.565" bestFit="true" customWidth="true" style="0"/>
     <col min="11" max="11" width="29.279" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="16.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="16.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="19" max="19" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="20" max="20" width="108.402" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="35.277" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="16.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="16" max="16" width="31.707" bestFit="true" customWidth="true" style="0"/>
+    <col min="17" max="17" width="16.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="18" max="18" width="25.851" bestFit="true" customWidth="true" style="0"/>
+    <col min="19" max="19" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="20" max="20" width="22.28" bestFit="true" customWidth="true" style="0"/>
+    <col min="21" max="21" width="108.402" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" customHeight="1" ht="30">
+    <row r="1" spans="1:21" customHeight="1" ht="30">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -699,7 +766,7 @@
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
@@ -723,250 +790,271 @@
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:20">
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2">
         <v>9529368928</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" t="s">
         <v>27</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="N2" t="s">
         <v>28</v>
       </c>
-      <c r="T2" t="s">
+      <c r="P2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="1:20">
+      <c r="R2" t="s">
+        <v>30</v>
+      </c>
+      <c r="U2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G3">
         <v>9356155617</v>
       </c>
       <c r="H3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N3" t="s">
+        <v>35</v>
+      </c>
+      <c r="P3" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" t="s">
+        <v>30</v>
+      </c>
+      <c r="U3" t="s">
         <v>31</v>
       </c>
-      <c r="M3" t="s">
-        <v>32</v>
-      </c>
-      <c r="O3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>28</v>
-      </c>
-      <c r="T3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20">
+    </row>
+    <row r="4" spans="1:21">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G4">
         <v>9767689897</v>
       </c>
       <c r="H4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="K4">
         <v>16200</v>
       </c>
       <c r="L4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="M4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20">
+        <v>40</v>
+      </c>
+      <c r="N4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G5">
         <v>9923688716</v>
       </c>
       <c r="H5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="M5" t="s">
-        <v>39</v>
-      </c>
-      <c r="O5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>41</v>
-      </c>
-      <c r="T5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20">
+        <v>43</v>
+      </c>
+      <c r="N5" t="s">
+        <v>44</v>
+      </c>
+      <c r="P5" t="s">
+        <v>45</v>
+      </c>
+      <c r="R5" t="s">
+        <v>46</v>
+      </c>
+      <c r="U5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G6">
         <v>8677867777</v>
       </c>
       <c r="H6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="K6">
         <v>16200</v>
       </c>
       <c r="L6" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="M6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O6" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q6" t="s">
+        <v>40</v>
+      </c>
+      <c r="N6" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:20">
+      <c r="P6" t="s">
+        <v>49</v>
+      </c>
+      <c r="R6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G7">
         <v>9370401366</v>
       </c>
       <c r="H7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="K7">
         <v>16200</v>
       </c>
       <c r="L7" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="M7" t="s">
-        <v>32</v>
-      </c>
-      <c r="O7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20">
+        <v>34</v>
+      </c>
+      <c r="N7" t="s">
+        <v>35</v>
+      </c>
+      <c r="P7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G8">
         <v>6395064076</v>
       </c>
       <c r="H8" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="I8">
         <v>50</v>
@@ -975,433 +1063,472 @@
         <v>8100</v>
       </c>
       <c r="L8" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="M8" t="s">
-        <v>49</v>
-      </c>
-      <c r="O8" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>28</v>
-      </c>
-      <c r="T8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20">
+        <v>56</v>
+      </c>
+      <c r="N8" t="s">
+        <v>57</v>
+      </c>
+      <c r="P8" t="s">
+        <v>58</v>
+      </c>
+      <c r="R8" t="s">
+        <v>30</v>
+      </c>
+      <c r="U8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H9" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="K9">
         <v>12200</v>
       </c>
       <c r="L9" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="M9" t="s">
-        <v>55</v>
-      </c>
-      <c r="T9" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20">
+        <v>63</v>
+      </c>
+      <c r="N9" t="s">
+        <v>64</v>
+      </c>
+      <c r="U9" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G10">
         <v>7720870317</v>
       </c>
       <c r="H10" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="I10">
         <v>75</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="5">
         <v>2000</v>
       </c>
       <c r="L10" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="M10" t="s">
-        <v>55</v>
-      </c>
-      <c r="T10" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20">
+        <v>27</v>
+      </c>
+      <c r="N10" t="s">
+        <v>64</v>
+      </c>
+      <c r="U10" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H11" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="K11">
         <v>16200</v>
       </c>
       <c r="L11" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="M11" t="s">
-        <v>55</v>
-      </c>
-      <c r="T11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20">
+        <v>63</v>
+      </c>
+      <c r="N11" t="s">
+        <v>64</v>
+      </c>
+      <c r="U11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G12">
         <v>9975609853</v>
       </c>
       <c r="H12" t="s">
-        <v>35</v>
-      </c>
-      <c r="K12" s="4">
+        <v>38</v>
+      </c>
+      <c r="K12" s="5">
         <v>7000</v>
       </c>
       <c r="L12" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="M12" t="s">
-        <v>26</v>
-      </c>
-      <c r="T12" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20">
+        <v>27</v>
+      </c>
+      <c r="N12" t="s">
+        <v>28</v>
+      </c>
+      <c r="U12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H13" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="K13">
         <v>16200</v>
       </c>
       <c r="L13" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="M13" t="s">
-        <v>55</v>
-      </c>
-      <c r="T13" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20">
+        <v>63</v>
+      </c>
+      <c r="N13" t="s">
+        <v>64</v>
+      </c>
+      <c r="U13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="D14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G14">
         <v>8767223103</v>
       </c>
       <c r="H14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L14" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="M14" t="s">
-        <v>49</v>
-      </c>
-      <c r="T14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20">
+        <v>56</v>
+      </c>
+      <c r="N14" t="s">
+        <v>57</v>
+      </c>
+      <c r="U14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H15" t="s">
-        <v>35</v>
-      </c>
-      <c r="K15" s="4">
+        <v>38</v>
+      </c>
+      <c r="K15" s="5">
         <v>9450</v>
       </c>
       <c r="L15" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="M15" t="s">
-        <v>49</v>
-      </c>
-      <c r="T15" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20">
+        <v>56</v>
+      </c>
+      <c r="N15" t="s">
+        <v>57</v>
+      </c>
+      <c r="U15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="E16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G16">
         <v>9923355136</v>
       </c>
       <c r="H16" t="s">
+        <v>38</v>
+      </c>
+      <c r="K16" s="5">
+        <v>5000</v>
+      </c>
+      <c r="L16" t="s">
+        <v>84</v>
+      </c>
+      <c r="M16" t="s">
+        <v>34</v>
+      </c>
+      <c r="N16" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="4">
-        <v>5000</v>
-      </c>
-      <c r="L16" t="s">
-        <v>31</v>
-      </c>
-      <c r="M16" t="s">
-        <v>32</v>
-      </c>
-      <c r="O16" t="s">
-        <v>45</v>
-      </c>
-      <c r="T16" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20">
+      <c r="P16" t="s">
+        <v>52</v>
+      </c>
+      <c r="U16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="E17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G17">
         <v>9975074600</v>
       </c>
       <c r="H17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L17" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="M17" t="s">
-        <v>49</v>
-      </c>
-      <c r="T17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20">
+        <v>56</v>
+      </c>
+      <c r="N17" t="s">
+        <v>57</v>
+      </c>
+      <c r="U17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="E18" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G18">
         <v>9834614015</v>
       </c>
       <c r="H18" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="I18">
         <v>25</v>
       </c>
       <c r="L18" t="s">
-        <v>48</v>
+        <v>89</v>
       </c>
       <c r="M18" t="s">
-        <v>49</v>
-      </c>
-      <c r="O18" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>28</v>
-      </c>
-      <c r="T18" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20">
+        <v>56</v>
+      </c>
+      <c r="N18" t="s">
+        <v>57</v>
+      </c>
+      <c r="P18" t="s">
+        <v>90</v>
+      </c>
+      <c r="R18" t="s">
+        <v>30</v>
+      </c>
+      <c r="U18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="E19" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G19">
         <v>9529295079</v>
       </c>
       <c r="H19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="K19">
         <v>12200</v>
       </c>
       <c r="L19" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="M19" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20">
+        <v>94</v>
+      </c>
+      <c r="N19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D20" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="E20" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F20" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G20">
         <v>7420930118</v>
       </c>
       <c r="H20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L20" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="M20" t="s">
-        <v>26</v>
-      </c>
-      <c r="O20" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>79</v>
-      </c>
-      <c r="T20" t="s">
-        <v>29</v>
+        <v>40</v>
+      </c>
+      <c r="N20" t="s">
+        <v>28</v>
+      </c>
+      <c r="P20" t="s">
+        <v>97</v>
+      </c>
+      <c r="R20" t="s">
+        <v>98</v>
+      </c>
+      <c r="U20" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>